<commit_message>
Rewrite cleaning and portfolio notebooks - fix MV optimization and stale filter
</commit_message>
<xml_diff>
--- a/data_clean/stale_flags.xlsx
+++ b/data_clean/stale_flags.xlsx
@@ -930,7 +930,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.06430868167202572</v>
+        <v>0</v>
       </c>
       <c r="D28" t="b">
         <v>0</v>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.06389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D40" t="b">
         <v>0</v>
@@ -1236,7 +1236,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.009584664536741214</v>
+        <v>0.006430868167202572</v>
       </c>
       <c r="D45" t="b">
         <v>0</v>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0.1018867924528302</v>
+        <v>0</v>
       </c>
       <c r="D57" t="b">
         <v>0</v>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0.268370607028754</v>
+        <v>0.02202643171806168</v>
       </c>
       <c r="D63" t="b">
         <v>0</v>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.08945686900958466</v>
+        <v>0</v>
       </c>
       <c r="D68" t="b">
         <v>0</v>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>0.1086261980830671</v>
+        <v>0</v>
       </c>
       <c r="D71" t="b">
         <v>0</v>
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>0.08945686900958466</v>
+        <v>0</v>
       </c>
       <c r="D77" t="b">
         <v>0</v>
@@ -2118,7 +2118,7 @@
         </is>
       </c>
       <c r="C94" t="n">
-        <v>0.07028753993610223</v>
+        <v>0</v>
       </c>
       <c r="D94" t="b">
         <v>0</v>
@@ -2154,7 +2154,7 @@
         </is>
       </c>
       <c r="C96" t="n">
-        <v>0.2204472843450479</v>
+        <v>0.008130081300813009</v>
       </c>
       <c r="D96" t="b">
         <v>0</v>
@@ -2568,7 +2568,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.02489626556016597</v>
       </c>
       <c r="D119" t="b">
         <v>0</v>
@@ -2730,10 +2730,10 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>0.8019169329073482</v>
+        <v>0.07017543859649122</v>
       </c>
       <c r="D128" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="129">
@@ -2892,7 +2892,7 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>0.15</v>
+        <v>0.004901960784313725</v>
       </c>
       <c r="D137" t="b">
         <v>0</v>
@@ -2946,7 +2946,7 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>0.07028753993610223</v>
+        <v>0.03355704697986577</v>
       </c>
       <c r="D140" t="b">
         <v>0</v>
@@ -3108,7 +3108,7 @@
         </is>
       </c>
       <c r="C149" t="n">
-        <v>0.01597444089456869</v>
+        <v>0</v>
       </c>
       <c r="D149" t="b">
         <v>0</v>
@@ -3144,7 +3144,7 @@
         </is>
       </c>
       <c r="C151" t="n">
-        <v>0.2008547008547009</v>
+        <v>0</v>
       </c>
       <c r="D151" t="b">
         <v>0</v>
@@ -3198,7 +3198,7 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>0.009584664536741214</v>
+        <v>0</v>
       </c>
       <c r="D154" t="b">
         <v>0</v>
@@ -3306,7 +3306,7 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>0.196652719665272</v>
+        <v>0.005154639175257732</v>
       </c>
       <c r="D160" t="b">
         <v>0</v>
@@ -3846,7 +3846,7 @@
         </is>
       </c>
       <c r="C190" t="n">
-        <v>0.01916932907348243</v>
+        <v>0</v>
       </c>
       <c r="D190" t="b">
         <v>0</v>
@@ -4044,7 +4044,7 @@
         </is>
       </c>
       <c r="C201" t="n">
-        <v>0.06389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D201" t="b">
         <v>0</v>
@@ -4602,7 +4602,7 @@
         </is>
       </c>
       <c r="C232" t="n">
-        <v>0.1086261980830671</v>
+        <v>0</v>
       </c>
       <c r="D232" t="b">
         <v>0</v>
@@ -4854,7 +4854,7 @@
         </is>
       </c>
       <c r="C246" t="n">
-        <v>0.1086261980830671</v>
+        <v>0</v>
       </c>
       <c r="D246" t="b">
         <v>0</v>
@@ -5052,7 +5052,7 @@
         </is>
       </c>
       <c r="C257" t="n">
-        <v>0.1022364217252396</v>
+        <v>0</v>
       </c>
       <c r="D257" t="b">
         <v>0</v>
@@ -5178,7 +5178,7 @@
         </is>
       </c>
       <c r="C264" t="n">
-        <v>0.006389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D264" t="b">
         <v>0</v>
@@ -5700,10 +5700,10 @@
         </is>
       </c>
       <c r="C293" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.05263157894736842</v>
       </c>
       <c r="D293" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="294">
@@ -5736,7 +5736,7 @@
         </is>
       </c>
       <c r="C295" t="n">
-        <v>0.2912087912087912</v>
+        <v>0.07971014492753623</v>
       </c>
       <c r="D295" t="b">
         <v>0</v>
@@ -5772,7 +5772,7 @@
         </is>
       </c>
       <c r="C297" t="n">
-        <v>0.07667731629392971</v>
+        <v>0.00684931506849315</v>
       </c>
       <c r="D297" t="b">
         <v>0</v>
@@ -5790,7 +5790,7 @@
         </is>
       </c>
       <c r="C298" t="n">
-        <v>0.345360824742268</v>
+        <v>0.0310077519379845</v>
       </c>
       <c r="D298" t="b">
         <v>0</v>
@@ -5826,7 +5826,7 @@
         </is>
       </c>
       <c r="C300" t="n">
-        <v>0.0653061224489796</v>
+        <v>0.05785123966942149</v>
       </c>
       <c r="D300" t="b">
         <v>0</v>
@@ -5880,7 +5880,7 @@
         </is>
       </c>
       <c r="C303" t="n">
-        <v>0.125</v>
+        <v>0</v>
       </c>
       <c r="D303" t="b">
         <v>0</v>
@@ -5916,7 +5916,7 @@
         </is>
       </c>
       <c r="C305" t="n">
-        <v>0.05405405405405406</v>
+        <v>0.02787456445993031</v>
       </c>
       <c r="D305" t="b">
         <v>0</v>
@@ -5934,7 +5934,7 @@
         </is>
       </c>
       <c r="C306" t="n">
-        <v>0.1191709844559585</v>
+        <v>0.08743169398907104</v>
       </c>
       <c r="D306" t="b">
         <v>0</v>
@@ -6042,7 +6042,7 @@
         </is>
       </c>
       <c r="C312" t="n">
-        <v>0.164021164021164</v>
+        <v>0.08875739644970414</v>
       </c>
       <c r="D312" t="b">
         <v>0</v>
@@ -7140,7 +7140,7 @@
         </is>
       </c>
       <c r="C373" t="n">
-        <v>0.1565495207667732</v>
+        <v>0.003759398496240601</v>
       </c>
       <c r="D373" t="b">
         <v>0</v>
@@ -7230,7 +7230,7 @@
         </is>
       </c>
       <c r="C378" t="n">
-        <v>0.09584664536741214</v>
+        <v>0</v>
       </c>
       <c r="D378" t="b">
         <v>0</v>
@@ -7950,7 +7950,7 @@
         </is>
       </c>
       <c r="C418" t="n">
-        <v>0.05750798722044728</v>
+        <v>0</v>
       </c>
       <c r="D418" t="b">
         <v>0</v>
@@ -8022,7 +8022,7 @@
         </is>
       </c>
       <c r="C422" t="n">
-        <v>0.1022364217252396</v>
+        <v>0</v>
       </c>
       <c r="D422" t="b">
         <v>0</v>
@@ -8310,7 +8310,7 @@
         </is>
       </c>
       <c r="C438" t="n">
-        <v>0.05111821086261981</v>
+        <v>0</v>
       </c>
       <c r="D438" t="b">
         <v>0</v>
@@ -8724,7 +8724,7 @@
         </is>
       </c>
       <c r="C461" t="n">
-        <v>0.02875399361022364</v>
+        <v>0</v>
       </c>
       <c r="D461" t="b">
         <v>0</v>
@@ -8940,7 +8940,7 @@
         </is>
       </c>
       <c r="C473" t="n">
-        <v>0.1274131274131274</v>
+        <v>0</v>
       </c>
       <c r="D473" t="b">
         <v>0</v>
@@ -8958,7 +8958,7 @@
         </is>
       </c>
       <c r="C474" t="n">
-        <v>0.01597444089456869</v>
+        <v>0</v>
       </c>
       <c r="D474" t="b">
         <v>0</v>
@@ -8994,7 +8994,7 @@
         </is>
       </c>
       <c r="C476" t="n">
-        <v>0.2671009771986971</v>
+        <v>0.01762114537444934</v>
       </c>
       <c r="D476" t="b">
         <v>0</v>
@@ -9102,7 +9102,7 @@
         </is>
       </c>
       <c r="C482" t="n">
-        <v>0.1469648562300319</v>
+        <v>0</v>
       </c>
       <c r="D482" t="b">
         <v>0</v>
@@ -9192,7 +9192,7 @@
         </is>
       </c>
       <c r="C487" t="n">
-        <v>0.07028753993610223</v>
+        <v>0</v>
       </c>
       <c r="D487" t="b">
         <v>0</v>
@@ -9444,7 +9444,7 @@
         </is>
       </c>
       <c r="C501" t="n">
-        <v>0.1501597444089457</v>
+        <v>0</v>
       </c>
       <c r="D501" t="b">
         <v>0</v>
@@ -9714,7 +9714,7 @@
         </is>
       </c>
       <c r="C516" t="n">
-        <v>0.1405750798722045</v>
+        <v>0</v>
       </c>
       <c r="D516" t="b">
         <v>0</v>
@@ -10416,7 +10416,7 @@
         </is>
       </c>
       <c r="C555" t="n">
-        <v>0.1363636363636364</v>
+        <v>0</v>
       </c>
       <c r="D555" t="b">
         <v>0</v>
@@ -10578,7 +10578,7 @@
         </is>
       </c>
       <c r="C564" t="n">
-        <v>0.2300319488817891</v>
+        <v>0</v>
       </c>
       <c r="D564" t="b">
         <v>0</v>
@@ -10812,7 +10812,7 @@
         </is>
       </c>
       <c r="C577" t="n">
-        <v>0.1277955271565495</v>
+        <v>0</v>
       </c>
       <c r="D577" t="b">
         <v>0</v>
@@ -10938,7 +10938,7 @@
         </is>
       </c>
       <c r="C584" t="n">
-        <v>0.1309904153354633</v>
+        <v>0</v>
       </c>
       <c r="D584" t="b">
         <v>0</v>
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="C588" t="n">
-        <v>0.06389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D588" t="b">
         <v>0</v>
@@ -11190,7 +11190,7 @@
         </is>
       </c>
       <c r="C598" t="n">
-        <v>0.1086261980830671</v>
+        <v>0</v>
       </c>
       <c r="D598" t="b">
         <v>0</v>
@@ -11280,7 +11280,7 @@
         </is>
       </c>
       <c r="C603" t="n">
-        <v>0.006389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D603" t="b">
         <v>0</v>
@@ -11352,7 +11352,7 @@
         </is>
       </c>
       <c r="C607" t="n">
-        <v>0.1277955271565495</v>
+        <v>0</v>
       </c>
       <c r="D607" t="b">
         <v>0</v>
@@ -11514,7 +11514,7 @@
         </is>
       </c>
       <c r="C616" t="n">
-        <v>0.01277955271565495</v>
+        <v>0</v>
       </c>
       <c r="D616" t="b">
         <v>0</v>
@@ -11586,7 +11586,7 @@
         </is>
       </c>
       <c r="C620" t="n">
-        <v>0.1437699680511182</v>
+        <v>0</v>
       </c>
       <c r="D620" t="b">
         <v>0</v>
@@ -11676,7 +11676,7 @@
         </is>
       </c>
       <c r="C625" t="n">
-        <v>0.1309904153354633</v>
+        <v>0</v>
       </c>
       <c r="D625" t="b">
         <v>0</v>
@@ -11694,7 +11694,7 @@
         </is>
       </c>
       <c r="C626" t="n">
-        <v>0.134185303514377</v>
+        <v>0</v>
       </c>
       <c r="D626" t="b">
         <v>0</v>
@@ -11856,7 +11856,7 @@
         </is>
       </c>
       <c r="C635" t="n">
-        <v>0.1246006389776358</v>
+        <v>0</v>
       </c>
       <c r="D635" t="b">
         <v>0</v>
@@ -12000,7 +12000,7 @@
         </is>
       </c>
       <c r="C643" t="n">
-        <v>0.1182108626198083</v>
+        <v>0</v>
       </c>
       <c r="D643" t="b">
         <v>0</v>
@@ -12054,7 +12054,7 @@
         </is>
       </c>
       <c r="C646" t="n">
-        <v>0.07028753993610223</v>
+        <v>0</v>
       </c>
       <c r="D646" t="b">
         <v>0</v>
@@ -12180,7 +12180,7 @@
         </is>
       </c>
       <c r="C653" t="n">
-        <v>0.03833865814696485</v>
+        <v>0</v>
       </c>
       <c r="D653" t="b">
         <v>0</v>
@@ -12324,7 +12324,7 @@
         </is>
       </c>
       <c r="C661" t="n">
-        <v>0.134185303514377</v>
+        <v>0</v>
       </c>
       <c r="D661" t="b">
         <v>0</v>
@@ -12432,7 +12432,7 @@
         </is>
       </c>
       <c r="C667" t="n">
-        <v>0.08223684210526316</v>
+        <v>0</v>
       </c>
       <c r="D667" t="b">
         <v>0</v>
@@ -12558,7 +12558,7 @@
         </is>
       </c>
       <c r="C674" t="n">
-        <v>0.07432432432432433</v>
+        <v>0</v>
       </c>
       <c r="D674" t="b">
         <v>0</v>
@@ -12828,7 +12828,7 @@
         </is>
       </c>
       <c r="C689" t="n">
-        <v>0.03194888178913738</v>
+        <v>0</v>
       </c>
       <c r="D689" t="b">
         <v>0</v>
@@ -12900,7 +12900,7 @@
         </is>
       </c>
       <c r="C693" t="n">
-        <v>0.09375</v>
+        <v>0</v>
       </c>
       <c r="D693" t="b">
         <v>0</v>
@@ -13080,7 +13080,7 @@
         </is>
       </c>
       <c r="C703" t="n">
-        <v>0.05394190871369295</v>
+        <v>0</v>
       </c>
       <c r="D703" t="b">
         <v>0</v>
@@ -13134,7 +13134,7 @@
         </is>
       </c>
       <c r="C706" t="n">
-        <v>0.08306709265175719</v>
+        <v>0</v>
       </c>
       <c r="D706" t="b">
         <v>0</v>
@@ -13206,7 +13206,7 @@
         </is>
       </c>
       <c r="C710" t="n">
-        <v>0.08945686900958466</v>
+        <v>0</v>
       </c>
       <c r="D710" t="b">
         <v>0</v>
@@ -13260,7 +13260,7 @@
         </is>
       </c>
       <c r="C713" t="n">
-        <v>0.1731601731601732</v>
+        <v>0</v>
       </c>
       <c r="D713" t="b">
         <v>0</v>
@@ -13404,7 +13404,7 @@
         </is>
       </c>
       <c r="C721" t="n">
-        <v>0.03833865814696485</v>
+        <v>0</v>
       </c>
       <c r="D721" t="b">
         <v>0</v>
@@ -13602,7 +13602,7 @@
         </is>
       </c>
       <c r="C732" t="n">
-        <v>0.02236421725239617</v>
+        <v>0</v>
       </c>
       <c r="D732" t="b">
         <v>0</v>
@@ -13836,7 +13836,7 @@
         </is>
       </c>
       <c r="C745" t="n">
-        <v>0.1405750798722045</v>
+        <v>0</v>
       </c>
       <c r="D745" t="b">
         <v>0</v>
@@ -13908,7 +13908,7 @@
         </is>
       </c>
       <c r="C749" t="n">
-        <v>0.1533546325878594</v>
+        <v>0</v>
       </c>
       <c r="D749" t="b">
         <v>0</v>
@@ -13962,7 +13962,7 @@
         </is>
       </c>
       <c r="C752" t="n">
-        <v>0.1469648562300319</v>
+        <v>0</v>
       </c>
       <c r="D752" t="b">
         <v>0</v>
@@ -14088,7 +14088,7 @@
         </is>
       </c>
       <c r="C759" t="n">
-        <v>0.05750798722044728</v>
+        <v>0</v>
       </c>
       <c r="D759" t="b">
         <v>0</v>
@@ -14178,7 +14178,7 @@
         </is>
       </c>
       <c r="C764" t="n">
-        <v>0.1491935483870968</v>
+        <v>0</v>
       </c>
       <c r="D764" t="b">
         <v>0</v>
@@ -14214,7 +14214,7 @@
         </is>
       </c>
       <c r="C766" t="n">
-        <v>0.1565495207667732</v>
+        <v>0</v>
       </c>
       <c r="D766" t="b">
         <v>0</v>
@@ -14268,7 +14268,7 @@
         </is>
       </c>
       <c r="C769" t="n">
-        <v>0.1054313099041534</v>
+        <v>0</v>
       </c>
       <c r="D769" t="b">
         <v>0</v>
@@ -14304,7 +14304,7 @@
         </is>
       </c>
       <c r="C771" t="n">
-        <v>0.04472843450479233</v>
+        <v>0</v>
       </c>
       <c r="D771" t="b">
         <v>0</v>
@@ -14466,7 +14466,7 @@
         </is>
       </c>
       <c r="C780" t="n">
-        <v>0.0255591054313099</v>
+        <v>0</v>
       </c>
       <c r="D780" t="b">
         <v>0</v>
@@ -14556,7 +14556,7 @@
         </is>
       </c>
       <c r="C785" t="n">
-        <v>0.1264367816091954</v>
+        <v>0</v>
       </c>
       <c r="D785" t="b">
         <v>0</v>
@@ -14718,7 +14718,7 @@
         </is>
       </c>
       <c r="C794" t="n">
-        <v>0.1182108626198083</v>
+        <v>0</v>
       </c>
       <c r="D794" t="b">
         <v>0</v>
@@ -14790,7 +14790,7 @@
         </is>
       </c>
       <c r="C798" t="n">
-        <v>0.05431309904153354</v>
+        <v>0.02</v>
       </c>
       <c r="D798" t="b">
         <v>0</v>
@@ -15132,7 +15132,7 @@
         </is>
       </c>
       <c r="C817" t="n">
-        <v>0.003194888178913738</v>
+        <v>0</v>
       </c>
       <c r="D817" t="b">
         <v>0</v>
@@ -15690,7 +15690,7 @@
         </is>
       </c>
       <c r="C848" t="n">
-        <v>0.1789137380191693</v>
+        <v>0.07547169811320754</v>
       </c>
       <c r="D848" t="b">
         <v>0</v>
@@ -15808,10 +15808,10 @@
         </is>
       </c>
       <c r="C855" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D855" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="856">
@@ -15842,10 +15842,10 @@
         </is>
       </c>
       <c r="C857" t="n">
-        <v>0.6847826086956522</v>
+        <v>0.08771929824561403</v>
       </c>
       <c r="D857" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="858">
@@ -15892,7 +15892,7 @@
         </is>
       </c>
       <c r="C860" t="n">
-        <v>0.1351351351351351</v>
+        <v>0.0505050505050505</v>
       </c>
       <c r="D860" t="b">
         <v>0</v>
@@ -15974,10 +15974,10 @@
         </is>
       </c>
       <c r="C865" t="n">
-        <v>0.9862385321100917</v>
+        <v>0</v>
       </c>
       <c r="D865" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="866">
@@ -15992,7 +15992,7 @@
         </is>
       </c>
       <c r="C866" t="n">
-        <v>0.3298969072164948</v>
+        <v>0.05925925925925926</v>
       </c>
       <c r="D866" t="b">
         <v>0</v>
@@ -16042,10 +16042,10 @@
         </is>
       </c>
       <c r="C869" t="n">
-        <v>0.6327433628318584</v>
+        <v>0.0759493670886076</v>
       </c>
       <c r="D869" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="870">
@@ -16110,7 +16110,7 @@
         </is>
       </c>
       <c r="C873" t="n">
-        <v>0.2405063291139241</v>
+        <v>0.05084745762711865</v>
       </c>
       <c r="D873" t="b">
         <v>0</v>
@@ -16144,7 +16144,7 @@
         </is>
       </c>
       <c r="C875" t="n">
-        <v>0.06349206349206349</v>
+        <v>0.053475935828877</v>
       </c>
       <c r="D875" t="b">
         <v>0</v>
@@ -16412,7 +16412,7 @@
         </is>
       </c>
       <c r="C890" t="n">
-        <v>0.1209150326797386</v>
+        <v>0.01098901098901099</v>
       </c>
       <c r="D890" t="b">
         <v>0</v>
@@ -16520,7 +16520,7 @@
         </is>
       </c>
       <c r="C896" t="n">
-        <v>0.01277955271565495</v>
+        <v>0.009646302250803859</v>
       </c>
       <c r="D896" t="b">
         <v>0</v>
@@ -16844,7 +16844,7 @@
         </is>
       </c>
       <c r="C914" t="n">
-        <v>0.09904153354632587</v>
+        <v>0</v>
       </c>
       <c r="D914" t="b">
         <v>0</v>
@@ -16952,7 +16952,7 @@
         </is>
       </c>
       <c r="C920" t="n">
-        <v>0.07667731629392971</v>
+        <v>0</v>
       </c>
       <c r="D920" t="b">
         <v>0</v>
@@ -17006,7 +17006,7 @@
         </is>
       </c>
       <c r="C923" t="n">
-        <v>0.03194888178913738</v>
+        <v>0.006578947368421052</v>
       </c>
       <c r="D923" t="b">
         <v>0</v>
@@ -17096,7 +17096,7 @@
         </is>
       </c>
       <c r="C928" t="n">
-        <v>0.006389776357827476</v>
+        <v>0.003215434083601286</v>
       </c>
       <c r="D928" t="b">
         <v>0</v>
@@ -17150,10 +17150,10 @@
         </is>
       </c>
       <c r="C931" t="n">
-        <v>0.588477366255144</v>
+        <v>0.0101010101010101</v>
       </c>
       <c r="D931" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="932">
@@ -17168,7 +17168,7 @@
         </is>
       </c>
       <c r="C932" t="n">
-        <v>0.08163265306122448</v>
+        <v>0.01739130434782609</v>
       </c>
       <c r="D932" t="b">
         <v>0</v>
@@ -17348,7 +17348,7 @@
         </is>
       </c>
       <c r="C942" t="n">
-        <v>0.02875399361022364</v>
+        <v>0.006578947368421052</v>
       </c>
       <c r="D942" t="b">
         <v>0</v>
@@ -17420,7 +17420,7 @@
         </is>
       </c>
       <c r="C946" t="n">
-        <v>0.1309904153354633</v>
+        <v>0.02173913043478261</v>
       </c>
       <c r="D946" t="b">
         <v>0</v>
@@ -17546,7 +17546,7 @@
         </is>
       </c>
       <c r="C953" t="n">
-        <v>0.01597444089456869</v>
+        <v>0</v>
       </c>
       <c r="D953" t="b">
         <v>0</v>
@@ -17690,10 +17690,10 @@
         </is>
       </c>
       <c r="C961" t="n">
-        <v>0.7657657657657657</v>
+        <v>0</v>
       </c>
       <c r="D961" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="962">
@@ -17906,7 +17906,7 @@
         </is>
       </c>
       <c r="C973" t="n">
-        <v>0.02875399361022364</v>
+        <v>0</v>
       </c>
       <c r="D973" t="b">
         <v>0</v>
@@ -17960,10 +17960,10 @@
         </is>
       </c>
       <c r="C976" t="n">
-        <v>0.6092436974789915</v>
+        <v>0</v>
       </c>
       <c r="D976" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="977">
@@ -18068,7 +18068,7 @@
         </is>
       </c>
       <c r="C982" t="n">
-        <v>0.1274131274131274</v>
+        <v>0.008771929824561403</v>
       </c>
       <c r="D982" t="b">
         <v>0</v>
@@ -18176,7 +18176,7 @@
         </is>
       </c>
       <c r="C988" t="n">
-        <v>0.1054313099041534</v>
+        <v>0.003584229390681004</v>
       </c>
       <c r="D988" t="b">
         <v>0</v>
@@ -18212,7 +18212,7 @@
         </is>
       </c>
       <c r="C990" t="n">
-        <v>0.3761061946902655</v>
+        <v>0.0273972602739726</v>
       </c>
       <c r="D990" t="b">
         <v>0</v>
@@ -18356,7 +18356,7 @@
         </is>
       </c>
       <c r="C998" t="n">
-        <v>0.4133333333333333</v>
+        <v>0.02941176470588235</v>
       </c>
       <c r="D998" t="b">
         <v>0</v>
@@ -18428,7 +18428,7 @@
         </is>
       </c>
       <c r="C1002" t="n">
-        <v>0.02893890675241157</v>
+        <v>0.0131578947368421</v>
       </c>
       <c r="D1002" t="b">
         <v>0</v>
@@ -18518,7 +18518,7 @@
         </is>
       </c>
       <c r="C1007" t="n">
-        <v>0.1390728476821192</v>
+        <v>0</v>
       </c>
       <c r="D1007" t="b">
         <v>0</v>
@@ -18572,7 +18572,7 @@
         </is>
       </c>
       <c r="C1010" t="n">
-        <v>0.09904153354632587</v>
+        <v>0</v>
       </c>
       <c r="D1010" t="b">
         <v>0</v>
@@ -18734,7 +18734,7 @@
         </is>
       </c>
       <c r="C1019" t="n">
-        <v>0.121405750798722</v>
+        <v>0</v>
       </c>
       <c r="D1019" t="b">
         <v>0</v>
@@ -18788,7 +18788,7 @@
         </is>
       </c>
       <c r="C1022" t="n">
-        <v>0.06389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D1022" t="b">
         <v>0</v>
@@ -18860,7 +18860,7 @@
         </is>
       </c>
       <c r="C1026" t="n">
-        <v>0.1629392971246006</v>
+        <v>0.01515151515151515</v>
       </c>
       <c r="D1026" t="b">
         <v>0</v>
@@ -18878,7 +18878,7 @@
         </is>
       </c>
       <c r="C1027" t="n">
-        <v>0.3546325878594249</v>
+        <v>0</v>
       </c>
       <c r="D1027" t="b">
         <v>0</v>
@@ -18896,7 +18896,7 @@
         </is>
       </c>
       <c r="C1028" t="n">
-        <v>0.1751824817518248</v>
+        <v>0</v>
       </c>
       <c r="D1028" t="b">
         <v>0</v>
@@ -19058,7 +19058,7 @@
         </is>
       </c>
       <c r="C1037" t="n">
-        <v>0.1086261980830671</v>
+        <v>0.04166666666666666</v>
       </c>
       <c r="D1037" t="b">
         <v>0</v>
@@ -19274,7 +19274,7 @@
         </is>
       </c>
       <c r="C1049" t="n">
-        <v>0.06028368794326241</v>
+        <v>0.03272727272727273</v>
       </c>
       <c r="D1049" t="b">
         <v>0</v>
@@ -19310,7 +19310,7 @@
         </is>
       </c>
       <c r="C1051" t="n">
-        <v>0.07667731629392971</v>
+        <v>0.02040816326530612</v>
       </c>
       <c r="D1051" t="b">
         <v>0</v>
@@ -19364,10 +19364,10 @@
         </is>
       </c>
       <c r="C1054" t="n">
-        <v>0.7028753993610224</v>
+        <v>0.04123711340206185</v>
       </c>
       <c r="D1054" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1055">
@@ -19508,10 +19508,10 @@
         </is>
       </c>
       <c r="C1062" t="n">
-        <v>0.8296296296296296</v>
+        <v>0.04347826086956522</v>
       </c>
       <c r="D1062" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1063">
@@ -19598,10 +19598,10 @@
         </is>
       </c>
       <c r="C1067" t="n">
-        <v>0.9094650205761317</v>
+        <v>0.1481481481481481</v>
       </c>
       <c r="D1067" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1068">
@@ -19796,7 +19796,7 @@
         </is>
       </c>
       <c r="C1078" t="n">
-        <v>0.05111821086261981</v>
+        <v>0.04516129032258064</v>
       </c>
       <c r="D1078" t="b">
         <v>0</v>
@@ -19940,7 +19940,7 @@
         </is>
       </c>
       <c r="C1086" t="n">
-        <v>0.1757188498402556</v>
+        <v>0.05535055350553506</v>
       </c>
       <c r="D1086" t="b">
         <v>0</v>
@@ -19976,7 +19976,7 @@
         </is>
       </c>
       <c r="C1088" t="n">
-        <v>0.02875399361022364</v>
+        <v>0.02572347266881029</v>
       </c>
       <c r="D1088" t="b">
         <v>0</v>
@@ -20246,7 +20246,7 @@
         </is>
       </c>
       <c r="C1103" t="n">
-        <v>0.07987220447284345</v>
+        <v>0.04666666666666667</v>
       </c>
       <c r="D1103" t="b">
         <v>0</v>
@@ -20480,7 +20480,7 @@
         </is>
       </c>
       <c r="C1116" t="n">
-        <v>0.05118110236220472</v>
+        <v>0.04382470119521913</v>
       </c>
       <c r="D1116" t="b">
         <v>0</v>
@@ -20570,7 +20570,7 @@
         </is>
       </c>
       <c r="C1121" t="n">
-        <v>0.1373801916932907</v>
+        <v>0.05376344086021505</v>
       </c>
       <c r="D1121" t="b">
         <v>0</v>
@@ -20624,7 +20624,7 @@
         </is>
       </c>
       <c r="C1124" t="n">
-        <v>0.1694214876033058</v>
+        <v>0.0202020202020202</v>
       </c>
       <c r="D1124" t="b">
         <v>0</v>
@@ -20642,7 +20642,7 @@
         </is>
       </c>
       <c r="C1125" t="n">
-        <v>0.1182108626198083</v>
+        <v>0.05555555555555555</v>
       </c>
       <c r="D1125" t="b">
         <v>0</v>
@@ -20786,7 +20786,7 @@
         </is>
       </c>
       <c r="C1133" t="n">
-        <v>0.2523961661341853</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="D1133" t="b">
         <v>0</v>
@@ -20966,7 +20966,7 @@
         </is>
       </c>
       <c r="C1143" t="n">
-        <v>0.03833865814696485</v>
+        <v>0.0130718954248366</v>
       </c>
       <c r="D1143" t="b">
         <v>0</v>
@@ -21020,7 +21020,7 @@
         </is>
       </c>
       <c r="C1146" t="n">
-        <v>0.06389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D1146" t="b">
         <v>0</v>
@@ -21092,10 +21092,10 @@
         </is>
       </c>
       <c r="C1150" t="n">
-        <v>0.9504950495049505</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="D1150" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1151">
@@ -21128,7 +21128,7 @@
         </is>
       </c>
       <c r="C1152" t="n">
-        <v>0.121405750798722</v>
+        <v>0.06574394463667819</v>
       </c>
       <c r="D1152" t="b">
         <v>0</v>
@@ -21218,7 +21218,7 @@
         </is>
       </c>
       <c r="C1157" t="n">
-        <v>0.0255591054313099</v>
+        <v>0.01612903225806452</v>
       </c>
       <c r="D1157" t="b">
         <v>0</v>
@@ -21254,7 +21254,7 @@
         </is>
       </c>
       <c r="C1159" t="n">
-        <v>0.01597444089456869</v>
+        <v>0.003257328990228013</v>
       </c>
       <c r="D1159" t="b">
         <v>0</v>
@@ -21326,7 +21326,7 @@
         </is>
       </c>
       <c r="C1163" t="n">
-        <v>0.07667731629392971</v>
+        <v>0.0436241610738255</v>
       </c>
       <c r="D1163" t="b">
         <v>0</v>
@@ -21344,7 +21344,7 @@
         </is>
       </c>
       <c r="C1164" t="n">
-        <v>0.2177121771217712</v>
+        <v>0.05045871559633028</v>
       </c>
       <c r="D1164" t="b">
         <v>0</v>
@@ -21434,7 +21434,7 @@
         </is>
       </c>
       <c r="C1169" t="n">
-        <v>0.06037735849056604</v>
+        <v>0.04651162790697674</v>
       </c>
       <c r="D1169" t="b">
         <v>0</v>
@@ -21542,7 +21542,7 @@
         </is>
       </c>
       <c r="C1175" t="n">
-        <v>0.4651162790697674</v>
+        <v>0.04320987654320987</v>
       </c>
       <c r="D1175" t="b">
         <v>0</v>
@@ -21722,7 +21722,7 @@
         </is>
       </c>
       <c r="C1185" t="n">
-        <v>0.03928571428571428</v>
+        <v>0.01838235294117647</v>
       </c>
       <c r="D1185" t="b">
         <v>0</v>
@@ -21830,7 +21830,7 @@
         </is>
       </c>
       <c r="C1191" t="n">
-        <v>0.02875399361022364</v>
+        <v>0.01941747572815534</v>
       </c>
       <c r="D1191" t="b">
         <v>0</v>
@@ -21848,7 +21848,7 @@
         </is>
       </c>
       <c r="C1192" t="n">
-        <v>0.04472843450479233</v>
+        <v>0.02631578947368421</v>
       </c>
       <c r="D1192" t="b">
         <v>0</v>
@@ -21866,10 +21866,10 @@
         </is>
       </c>
       <c r="C1193" t="n">
-        <v>0.5910543130990416</v>
+        <v>0.03076923076923077</v>
       </c>
       <c r="D1193" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1194">
@@ -21992,7 +21992,7 @@
         </is>
       </c>
       <c r="C1200" t="n">
-        <v>0.05750798722044728</v>
+        <v>0.03311258278145696</v>
       </c>
       <c r="D1200" t="b">
         <v>0</v>
@@ -22010,7 +22010,7 @@
         </is>
       </c>
       <c r="C1201" t="n">
-        <v>0.05119453924914676</v>
+        <v>0.02464788732394366</v>
       </c>
       <c r="D1201" t="b">
         <v>0</v>
@@ -22046,7 +22046,7 @@
         </is>
       </c>
       <c r="C1203" t="n">
-        <v>0.103448275862069</v>
+        <v>0.0502092050209205</v>
       </c>
       <c r="D1203" t="b">
         <v>0</v>
@@ -22064,10 +22064,10 @@
         </is>
       </c>
       <c r="C1204" t="n">
-        <v>0.9839743589743589</v>
+        <v>0</v>
       </c>
       <c r="D1204" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1205">
@@ -22370,7 +22370,7 @@
         </is>
       </c>
       <c r="C1221" t="n">
-        <v>0.0926517571884984</v>
+        <v>0.01041666666666667</v>
       </c>
       <c r="D1221" t="b">
         <v>0</v>
@@ -22460,7 +22460,7 @@
         </is>
       </c>
       <c r="C1226" t="n">
-        <v>0.01916932907348243</v>
+        <v>0.01607717041800643</v>
       </c>
       <c r="D1226" t="b">
         <v>0</v>
@@ -22604,7 +22604,7 @@
         </is>
       </c>
       <c r="C1234" t="n">
-        <v>0.07348242811501597</v>
+        <v>0.06774193548387097</v>
       </c>
       <c r="D1234" t="b">
         <v>0</v>
@@ -22820,7 +22820,7 @@
         </is>
       </c>
       <c r="C1246" t="n">
-        <v>0.08791208791208792</v>
+        <v>0.06130268199233716</v>
       </c>
       <c r="D1246" t="b">
         <v>0</v>
@@ -23000,7 +23000,7 @@
         </is>
       </c>
       <c r="C1256" t="n">
-        <v>0.1789137380191693</v>
+        <v>0.01167315175097276</v>
       </c>
       <c r="D1256" t="b">
         <v>0</v>
@@ -23036,7 +23036,7 @@
         </is>
       </c>
       <c r="C1258" t="n">
-        <v>0.07348242811501597</v>
+        <v>0.0493421052631579</v>
       </c>
       <c r="D1258" t="b">
         <v>0</v>
@@ -23072,7 +23072,7 @@
         </is>
       </c>
       <c r="C1260" t="n">
-        <v>0.2608695652173913</v>
+        <v>0.1075268817204301</v>
       </c>
       <c r="D1260" t="b">
         <v>0</v>
@@ -23288,7 +23288,7 @@
         </is>
       </c>
       <c r="C1272" t="n">
-        <v>0.3961661341853035</v>
+        <v>0.07731958762886598</v>
       </c>
       <c r="D1272" t="b">
         <v>0</v>
@@ -23432,7 +23432,7 @@
         </is>
       </c>
       <c r="C1280" t="n">
-        <v>0.06228373702422145</v>
+        <v>0.05263157894736842</v>
       </c>
       <c r="D1280" t="b">
         <v>0</v>
@@ -23486,10 +23486,10 @@
         </is>
       </c>
       <c r="C1283" t="n">
-        <v>0.5343511450381679</v>
+        <v>0.08</v>
       </c>
       <c r="D1283" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1284">
@@ -23504,7 +23504,7 @@
         </is>
       </c>
       <c r="C1284" t="n">
-        <v>0.1789137380191693</v>
+        <v>0.09090909090909091</v>
       </c>
       <c r="D1284" t="b">
         <v>0</v>
@@ -23594,7 +23594,7 @@
         </is>
       </c>
       <c r="C1289" t="n">
-        <v>0.09584664536741214</v>
+        <v>0.02758620689655172</v>
       </c>
       <c r="D1289" t="b">
         <v>0</v>
@@ -23630,7 +23630,7 @@
         </is>
       </c>
       <c r="C1291" t="n">
-        <v>0.1277955271565495</v>
+        <v>0.007246376811594203</v>
       </c>
       <c r="D1291" t="b">
         <v>0</v>
@@ -23684,7 +23684,7 @@
         </is>
       </c>
       <c r="C1294" t="n">
-        <v>0.3099041533546326</v>
+        <v>0.06912442396313365</v>
       </c>
       <c r="D1294" t="b">
         <v>0</v>
@@ -23702,7 +23702,7 @@
         </is>
       </c>
       <c r="C1295" t="n">
-        <v>0.1884984025559105</v>
+        <v>0.0310077519379845</v>
       </c>
       <c r="D1295" t="b">
         <v>0</v>
@@ -23882,7 +23882,7 @@
         </is>
       </c>
       <c r="C1305" t="n">
-        <v>0.3194888178913738</v>
+        <v>0.1052631578947368</v>
       </c>
       <c r="D1305" t="b">
         <v>0</v>
@@ -23918,7 +23918,7 @@
         </is>
       </c>
       <c r="C1307" t="n">
-        <v>0.04472843450479233</v>
+        <v>0.04180064308681672</v>
       </c>
       <c r="D1307" t="b">
         <v>0</v>
@@ -24008,7 +24008,7 @@
         </is>
       </c>
       <c r="C1312" t="n">
-        <v>0.2492012779552716</v>
+        <v>0.08627450980392157</v>
       </c>
       <c r="D1312" t="b">
         <v>0</v>
@@ -24150,7 +24150,7 @@
         </is>
       </c>
       <c r="C1320" t="n">
-        <v>0.05119453924914676</v>
+        <v>0.02807017543859649</v>
       </c>
       <c r="D1320" t="b">
         <v>0</v>
@@ -24186,7 +24186,7 @@
         </is>
       </c>
       <c r="C1322" t="n">
-        <v>0.1150159744408946</v>
+        <v>0.03886925795053003</v>
       </c>
       <c r="D1322" t="b">
         <v>0</v>
@@ -24258,7 +24258,7 @@
         </is>
       </c>
       <c r="C1326" t="n">
-        <v>0.1118210862619808</v>
+        <v>0.03146853146853147</v>
       </c>
       <c r="D1326" t="b">
         <v>0</v>
@@ -24294,10 +24294,10 @@
         </is>
       </c>
       <c r="C1328" t="n">
-        <v>0.7730263157894737</v>
+        <v>0.1333333333333333</v>
       </c>
       <c r="D1328" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1329">
@@ -24384,7 +24384,7 @@
         </is>
       </c>
       <c r="C1333" t="n">
-        <v>0.1789137380191693</v>
+        <v>0.03065134099616858</v>
       </c>
       <c r="D1333" t="b">
         <v>0</v>
@@ -24402,10 +24402,10 @@
         </is>
       </c>
       <c r="C1334" t="n">
-        <v>0.9877049180327869</v>
+        <v>0.25</v>
       </c>
       <c r="D1334" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1335">
@@ -24528,10 +24528,10 @@
         </is>
       </c>
       <c r="C1341" t="n">
-        <v>0.996742671009772</v>
+        <v>0</v>
       </c>
       <c r="D1341" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1342">
@@ -24564,7 +24564,7 @@
         </is>
       </c>
       <c r="C1343" t="n">
-        <v>0.2523961661341853</v>
+        <v>0.08764940239043825</v>
       </c>
       <c r="D1343" t="b">
         <v>0</v>
@@ -24618,7 +24618,7 @@
         </is>
       </c>
       <c r="C1346" t="n">
-        <v>0.2525252525252525</v>
+        <v>0.05752212389380531</v>
       </c>
       <c r="D1346" t="b">
         <v>0</v>
@@ -24654,7 +24654,7 @@
         </is>
       </c>
       <c r="C1348" t="n">
-        <v>0.02875399361022364</v>
+        <v>0.02572347266881029</v>
       </c>
       <c r="D1348" t="b">
         <v>0</v>
@@ -24888,7 +24888,7 @@
         </is>
       </c>
       <c r="C1361" t="n">
-        <v>0.1916932907348243</v>
+        <v>0.06015037593984962</v>
       </c>
       <c r="D1361" t="b">
         <v>0</v>
@@ -24906,10 +24906,10 @@
         </is>
       </c>
       <c r="C1362" t="n">
-        <v>0.6538461538461539</v>
+        <v>0.1081081081081081</v>
       </c>
       <c r="D1362" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1363">
@@ -24960,7 +24960,7 @@
         </is>
       </c>
       <c r="C1365" t="n">
-        <v>0.1294498381877023</v>
+        <v>0.02545454545454546</v>
       </c>
       <c r="D1365" t="b">
         <v>0</v>
@@ -25014,7 +25014,7 @@
         </is>
       </c>
       <c r="C1368" t="n">
-        <v>0.1503267973856209</v>
+        <v>0.07526881720430108</v>
       </c>
       <c r="D1368" t="b">
         <v>0</v>
@@ -25086,7 +25086,7 @@
         </is>
       </c>
       <c r="C1372" t="n">
-        <v>0.3794642857142857</v>
+        <v>0.04861111111111111</v>
       </c>
       <c r="D1372" t="b">
         <v>0</v>
@@ -25104,7 +25104,7 @@
         </is>
       </c>
       <c r="C1373" t="n">
-        <v>0.2332268370607029</v>
+        <v>0.02459016393442623</v>
       </c>
       <c r="D1373" t="b">
         <v>0</v>
@@ -25122,7 +25122,7 @@
         </is>
       </c>
       <c r="C1374" t="n">
-        <v>0.07987220447284345</v>
+        <v>0.0103448275862069</v>
       </c>
       <c r="D1374" t="b">
         <v>0</v>
@@ -25190,7 +25190,7 @@
         </is>
       </c>
       <c r="C1378" t="n">
-        <v>0.05594405594405594</v>
+        <v>0.01824817518248175</v>
       </c>
       <c r="D1378" t="b">
         <v>0</v>
@@ -25296,10 +25296,10 @@
         </is>
       </c>
       <c r="C1384" t="n">
-        <v>0.6299212598425197</v>
+        <v>0.07777777777777778</v>
       </c>
       <c r="D1384" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1385">
@@ -25314,10 +25314,10 @@
         </is>
       </c>
       <c r="C1385" t="n">
-        <v>0.6829268292682927</v>
+        <v>0</v>
       </c>
       <c r="D1385" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1386">
@@ -25332,10 +25332,10 @@
         </is>
       </c>
       <c r="C1386" t="n">
-        <v>0.9680511182108626</v>
+        <v>0.1818181818181818</v>
       </c>
       <c r="D1386" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1387">
@@ -25350,7 +25350,7 @@
         </is>
       </c>
       <c r="C1387" t="n">
-        <v>0.04792332268370607</v>
+        <v>0.01</v>
       </c>
       <c r="D1387" t="b">
         <v>0</v>
@@ -25404,10 +25404,10 @@
         </is>
       </c>
       <c r="C1390" t="n">
-        <v>0.7099236641221374</v>
+        <v>0</v>
       </c>
       <c r="D1390" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1391">
@@ -25438,10 +25438,10 @@
         </is>
       </c>
       <c r="C1392" t="n">
-        <v>0.5317460317460317</v>
+        <v>0.0423728813559322</v>
       </c>
       <c r="D1392" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1393">
@@ -25456,7 +25456,7 @@
         </is>
       </c>
       <c r="C1393" t="n">
-        <v>0.07028753993610223</v>
+        <v>0.01712328767123288</v>
       </c>
       <c r="D1393" t="b">
         <v>0</v>
@@ -25474,7 +25474,7 @@
         </is>
       </c>
       <c r="C1394" t="n">
-        <v>0.121405750798722</v>
+        <v>0.01449275362318841</v>
       </c>
       <c r="D1394" t="b">
         <v>0</v>
@@ -25492,7 +25492,7 @@
         </is>
       </c>
       <c r="C1395" t="n">
-        <v>0.04182509505703422</v>
+        <v>0.01574803149606299</v>
       </c>
       <c r="D1395" t="b">
         <v>0</v>
@@ -25582,7 +25582,7 @@
         </is>
       </c>
       <c r="C1400" t="n">
-        <v>0.04153354632587859</v>
+        <v>0.01644736842105263</v>
       </c>
       <c r="D1400" t="b">
         <v>0</v>
@@ -25600,7 +25600,7 @@
         </is>
       </c>
       <c r="C1401" t="n">
-        <v>0.06083650190114068</v>
+        <v>0.04651162790697674</v>
       </c>
       <c r="D1401" t="b">
         <v>0</v>
@@ -25636,10 +25636,10 @@
         </is>
       </c>
       <c r="C1403" t="n">
-        <v>0.8225108225108225</v>
+        <v>0.02439024390243903</v>
       </c>
       <c r="D1403" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1404">
@@ -25672,7 +25672,7 @@
         </is>
       </c>
       <c r="C1405" t="n">
-        <v>0.04472843450479233</v>
+        <v>0.03571428571428571</v>
       </c>
       <c r="D1405" t="b">
         <v>0</v>
@@ -25690,7 +25690,7 @@
         </is>
       </c>
       <c r="C1406" t="n">
-        <v>0.2044728434504792</v>
+        <v>0.03125</v>
       </c>
       <c r="D1406" t="b">
         <v>0</v>
@@ -25708,7 +25708,7 @@
         </is>
       </c>
       <c r="C1407" t="n">
-        <v>0.1469648562300319</v>
+        <v>0.03284671532846715</v>
       </c>
       <c r="D1407" t="b">
         <v>0</v>
@@ -25726,7 +25726,7 @@
         </is>
       </c>
       <c r="C1408" t="n">
-        <v>0.06070287539936102</v>
+        <v>0.01677852348993289</v>
       </c>
       <c r="D1408" t="b">
         <v>0</v>
@@ -25744,7 +25744,7 @@
         </is>
       </c>
       <c r="C1409" t="n">
-        <v>0.02875399361022364</v>
+        <v>0.0226537216828479</v>
       </c>
       <c r="D1409" t="b">
         <v>0</v>
@@ -25762,7 +25762,7 @@
         </is>
       </c>
       <c r="C1410" t="n">
-        <v>0.134185303514377</v>
+        <v>0.04642857142857143</v>
       </c>
       <c r="D1410" t="b">
         <v>0</v>
@@ -25780,7 +25780,7 @@
         </is>
       </c>
       <c r="C1411" t="n">
-        <v>0.09584664536741214</v>
+        <v>0.03169014084507042</v>
       </c>
       <c r="D1411" t="b">
         <v>0</v>
@@ -25798,10 +25798,10 @@
         </is>
       </c>
       <c r="C1412" t="n">
-        <v>0.7688888888888888</v>
+        <v>0.06</v>
       </c>
       <c r="D1412" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1413">
@@ -25816,7 +25816,7 @@
         </is>
       </c>
       <c r="C1413" t="n">
-        <v>0.07169811320754717</v>
+        <v>0.02008032128514056</v>
       </c>
       <c r="D1413" t="b">
         <v>0</v>
@@ -25834,7 +25834,7 @@
         </is>
       </c>
       <c r="C1414" t="n">
-        <v>0.1592920353982301</v>
+        <v>0.07035175879396985</v>
       </c>
       <c r="D1414" t="b">
         <v>0</v>
@@ -25852,7 +25852,7 @@
         </is>
       </c>
       <c r="C1415" t="n">
-        <v>0.2380952380952381</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="D1415" t="b">
         <v>0</v>
@@ -25870,7 +25870,7 @@
         </is>
       </c>
       <c r="C1416" t="n">
-        <v>0.05063291139240506</v>
+        <v>0.02183406113537118</v>
       </c>
       <c r="D1416" t="b">
         <v>0</v>
@@ -25940,7 +25940,7 @@
         </is>
       </c>
       <c r="C1420" t="n">
-        <v>0.05947955390334572</v>
+        <v>0.03474903474903475</v>
       </c>
       <c r="D1420" t="b">
         <v>0</v>
@@ -25958,10 +25958,10 @@
         </is>
       </c>
       <c r="C1421" t="n">
-        <v>0.9821428571428571</v>
+        <v>0.25</v>
       </c>
       <c r="D1421" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1422">
@@ -25976,10 +25976,10 @@
         </is>
       </c>
       <c r="C1422" t="n">
-        <v>0.7991967871485943</v>
+        <v>0.04</v>
       </c>
       <c r="D1422" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1423">
@@ -26012,7 +26012,7 @@
         </is>
       </c>
       <c r="C1424" t="n">
-        <v>0.1789137380191693</v>
+        <v>0.0193050193050193</v>
       </c>
       <c r="D1424" t="b">
         <v>0</v>
@@ -26030,10 +26030,10 @@
         </is>
       </c>
       <c r="C1425" t="n">
-        <v>0.7107438016528925</v>
+        <v>0.02985074626865672</v>
       </c>
       <c r="D1425" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1426">
@@ -26048,7 +26048,7 @@
         </is>
       </c>
       <c r="C1426" t="n">
-        <v>0.05111821086261981</v>
+        <v>0.01333333333333333</v>
       </c>
       <c r="D1426" t="b">
         <v>0</v>
@@ -26082,7 +26082,7 @@
         </is>
       </c>
       <c r="C1428" t="n">
-        <v>0.2012779552715655</v>
+        <v>0.05405405405405406</v>
       </c>
       <c r="D1428" t="b">
         <v>0</v>
@@ -26152,10 +26152,10 @@
         </is>
       </c>
       <c r="C1432" t="n">
-        <v>0.8312236286919831</v>
+        <v>0.1351351351351351</v>
       </c>
       <c r="D1432" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1433">
@@ -26170,10 +26170,10 @@
         </is>
       </c>
       <c r="C1433" t="n">
-        <v>0.7455357142857143</v>
+        <v>0.06779661016949153</v>
       </c>
       <c r="D1433" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1434">
@@ -26204,10 +26204,10 @@
         </is>
       </c>
       <c r="C1435" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D1435" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1436">
@@ -26238,7 +26238,7 @@
         </is>
       </c>
       <c r="C1437" t="n">
-        <v>0.2158273381294964</v>
+        <v>0.1507936507936508</v>
       </c>
       <c r="D1437" t="b">
         <v>0</v>
@@ -26256,7 +26256,7 @@
         </is>
       </c>
       <c r="C1438" t="n">
-        <v>0.3429752066115703</v>
+        <v>0.0196078431372549</v>
       </c>
       <c r="D1438" t="b">
         <v>0</v>
@@ -26358,10 +26358,10 @@
         </is>
       </c>
       <c r="C1444" t="n">
-        <v>0.625</v>
+        <v>0.03191489361702127</v>
       </c>
       <c r="D1444" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1445">
@@ -26392,10 +26392,10 @@
         </is>
       </c>
       <c r="C1446" t="n">
-        <v>0.8879668049792531</v>
+        <v>0.1</v>
       </c>
       <c r="D1446" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1447">
@@ -26410,7 +26410,7 @@
         </is>
       </c>
       <c r="C1447" t="n">
-        <v>0.1188524590163934</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="D1447" t="b">
         <v>0</v>
@@ -26446,7 +26446,7 @@
         </is>
       </c>
       <c r="C1449" t="n">
-        <v>0.07883817427385892</v>
+        <v>0.01785714285714286</v>
       </c>
       <c r="D1449" t="b">
         <v>0</v>
@@ -26480,10 +26480,10 @@
         </is>
       </c>
       <c r="C1451" t="n">
-        <v>0.8264840182648402</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="D1451" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1452">
@@ -26498,7 +26498,7 @@
         </is>
       </c>
       <c r="C1452" t="n">
-        <v>0.0860655737704918</v>
+        <v>0.03111111111111111</v>
       </c>
       <c r="D1452" t="b">
         <v>0</v>
@@ -26516,10 +26516,10 @@
         </is>
       </c>
       <c r="C1453" t="n">
-        <v>0.8060344827586207</v>
+        <v>0.04444444444444445</v>
       </c>
       <c r="D1453" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1454">
@@ -26550,10 +26550,10 @@
         </is>
       </c>
       <c r="C1455" t="n">
-        <v>0.8865248226950354</v>
+        <v>0.06666666666666667</v>
       </c>
       <c r="D1455" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1456">
@@ -26584,10 +26584,10 @@
         </is>
       </c>
       <c r="C1457" t="n">
-        <v>0.6157024793388429</v>
+        <v>0.09900990099009901</v>
       </c>
       <c r="D1457" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1458">
@@ -26782,7 +26782,7 @@
         </is>
       </c>
       <c r="C1468" t="n">
-        <v>0.1455938697318008</v>
+        <v>0</v>
       </c>
       <c r="D1468" t="b">
         <v>0</v>
@@ -26980,7 +26980,7 @@
         </is>
       </c>
       <c r="C1479" t="n">
-        <v>0.2195121951219512</v>
+        <v>0.07462686567164178</v>
       </c>
       <c r="D1479" t="b">
         <v>0</v>
@@ -27250,7 +27250,7 @@
         </is>
       </c>
       <c r="C1494" t="n">
-        <v>0.4864864864864865</v>
+        <v>0.01470588235294118</v>
       </c>
       <c r="D1494" t="b">
         <v>0</v>
@@ -27844,7 +27844,7 @@
         </is>
       </c>
       <c r="C1527" t="n">
-        <v>0.08626198083067092</v>
+        <v>0.0103448275862069</v>
       </c>
       <c r="D1527" t="b">
         <v>0</v>
@@ -27934,7 +27934,7 @@
         </is>
       </c>
       <c r="C1532" t="n">
-        <v>0.04472843450479233</v>
+        <v>0.006622516556291391</v>
       </c>
       <c r="D1532" t="b">
         <v>0</v>
@@ -28042,7 +28042,7 @@
         </is>
       </c>
       <c r="C1538" t="n">
-        <v>0.1693290734824281</v>
+        <v>0.03422053231939164</v>
       </c>
       <c r="D1538" t="b">
         <v>0</v>
@@ -28582,7 +28582,7 @@
         </is>
       </c>
       <c r="C1568" t="n">
-        <v>0.01277955271565495</v>
+        <v>0</v>
       </c>
       <c r="D1568" t="b">
         <v>0</v>
@@ -28618,7 +28618,7 @@
         </is>
       </c>
       <c r="C1570" t="n">
-        <v>0.3067092651757188</v>
+        <v>0.04977375565610859</v>
       </c>
       <c r="D1570" t="b">
         <v>0</v>
@@ -28726,10 +28726,10 @@
         </is>
       </c>
       <c r="C1576" t="n">
-        <v>0.635593220338983</v>
+        <v>0.02272727272727273</v>
       </c>
       <c r="D1576" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1577">
@@ -28744,7 +28744,7 @@
         </is>
       </c>
       <c r="C1577" t="n">
-        <v>0.0670926517571885</v>
+        <v>0.003412969283276451</v>
       </c>
       <c r="D1577" t="b">
         <v>0</v>
@@ -28798,7 +28798,7 @@
         </is>
       </c>
       <c r="C1580" t="n">
-        <v>0.255591054313099</v>
+        <v>0.008474576271186441</v>
       </c>
       <c r="D1580" t="b">
         <v>0</v>
@@ -29248,7 +29248,7 @@
         </is>
       </c>
       <c r="C1605" t="n">
-        <v>0.006389776357827476</v>
+        <v>0.003215434083601286</v>
       </c>
       <c r="D1605" t="b">
         <v>0</v>
@@ -29338,7 +29338,7 @@
         </is>
       </c>
       <c r="C1610" t="n">
-        <v>0.1693290734824281</v>
+        <v>0.03358208955223881</v>
       </c>
       <c r="D1610" t="b">
         <v>0</v>
@@ -29428,7 +29428,7 @@
         </is>
       </c>
       <c r="C1615" t="n">
-        <v>0.03194888178913738</v>
+        <v>0.009868421052631578</v>
       </c>
       <c r="D1615" t="b">
         <v>0</v>
@@ -29626,7 +29626,7 @@
         </is>
       </c>
       <c r="C1626" t="n">
-        <v>0.1075697211155379</v>
+        <v>0</v>
       </c>
       <c r="D1626" t="b">
         <v>0</v>
@@ -29680,7 +29680,7 @@
         </is>
       </c>
       <c r="C1629" t="n">
-        <v>0.1740890688259109</v>
+        <v>0</v>
       </c>
       <c r="D1629" t="b">
         <v>0</v>
@@ -29734,7 +29734,7 @@
         </is>
       </c>
       <c r="C1632" t="n">
-        <v>0.1646090534979424</v>
+        <v>0</v>
       </c>
       <c r="D1632" t="b">
         <v>0</v>
@@ -29932,7 +29932,7 @@
         </is>
       </c>
       <c r="C1643" t="n">
-        <v>0.06872852233676977</v>
+        <v>0</v>
       </c>
       <c r="D1643" t="b">
         <v>0</v>
@@ -29950,7 +29950,7 @@
         </is>
       </c>
       <c r="C1644" t="n">
-        <v>0.3623853211009174</v>
+        <v>0.01408450704225352</v>
       </c>
       <c r="D1644" t="b">
         <v>0</v>
@@ -29968,7 +29968,7 @@
         </is>
       </c>
       <c r="C1645" t="n">
-        <v>0.0707395498392283</v>
+        <v>0.00684931506849315</v>
       </c>
       <c r="D1645" t="b">
         <v>0</v>
@@ -29986,7 +29986,7 @@
         </is>
       </c>
       <c r="C1646" t="n">
-        <v>0.0670926517571885</v>
+        <v>0.003401360544217687</v>
       </c>
       <c r="D1646" t="b">
         <v>0</v>
@@ -30004,7 +30004,7 @@
         </is>
       </c>
       <c r="C1647" t="n">
-        <v>0.06389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D1647" t="b">
         <v>0</v>
@@ -30022,7 +30022,7 @@
         </is>
       </c>
       <c r="C1648" t="n">
-        <v>0.06389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D1648" t="b">
         <v>0</v>
@@ -30040,7 +30040,7 @@
         </is>
       </c>
       <c r="C1649" t="n">
-        <v>0.0726643598615917</v>
+        <v>0.003703703703703704</v>
       </c>
       <c r="D1649" t="b">
         <v>0</v>
@@ -30058,7 +30058,7 @@
         </is>
       </c>
       <c r="C1650" t="n">
-        <v>0.08097165991902834</v>
+        <v>0</v>
       </c>
       <c r="D1650" t="b">
         <v>0</v>
@@ -30076,7 +30076,7 @@
         </is>
       </c>
       <c r="C1651" t="n">
-        <v>0.06389776357827476</v>
+        <v>0</v>
       </c>
       <c r="D1651" t="b">
         <v>0</v>
@@ -30094,7 +30094,7 @@
         </is>
       </c>
       <c r="C1652" t="n">
-        <v>0.08333333333333333</v>
+        <v>0</v>
       </c>
       <c r="D1652" t="b">
         <v>0</v>
@@ -30112,7 +30112,7 @@
         </is>
       </c>
       <c r="C1653" t="n">
-        <v>0.3111111111111111</v>
+        <v>0.0392156862745098</v>
       </c>
       <c r="D1653" t="b">
         <v>0</v>
@@ -30130,7 +30130,7 @@
         </is>
       </c>
       <c r="C1654" t="n">
-        <v>0.08300395256916997</v>
+        <v>0.004273504273504274</v>
       </c>
       <c r="D1654" t="b">
         <v>0</v>
@@ -30148,7 +30148,7 @@
         </is>
       </c>
       <c r="C1655" t="n">
-        <v>0.1318181818181818</v>
+        <v>0.02072538860103627</v>
       </c>
       <c r="D1655" t="b">
         <v>0</v>
@@ -30166,7 +30166,7 @@
         </is>
       </c>
       <c r="C1656" t="n">
-        <v>0.1068376068376068</v>
+        <v>0.02325581395348837</v>
       </c>
       <c r="D1656" t="b">
         <v>0</v>
@@ -30184,10 +30184,10 @@
         </is>
       </c>
       <c r="C1657" t="n">
-        <v>0.5089285714285714</v>
+        <v>0.04504504504504504</v>
       </c>
       <c r="D1657" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1658">
@@ -30202,7 +30202,7 @@
         </is>
       </c>
       <c r="C1658" t="n">
-        <v>0.2311320754716981</v>
+        <v>0.07017543859649122</v>
       </c>
       <c r="D1658" t="b">
         <v>0</v>
@@ -30616,7 +30616,7 @@
         </is>
       </c>
       <c r="C1681" t="n">
-        <v>0.1980830670926517</v>
+        <v>0.03088803088803089</v>
       </c>
       <c r="D1681" t="b">
         <v>0</v>
@@ -30742,10 +30742,10 @@
         </is>
       </c>
       <c r="C1688" t="n">
-        <v>0.5775577557755776</v>
+        <v>0</v>
       </c>
       <c r="D1688" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1689">
@@ -30778,7 +30778,7 @@
         </is>
       </c>
       <c r="C1690" t="n">
-        <v>0.121405750798722</v>
+        <v>0</v>
       </c>
       <c r="D1690" t="b">
         <v>0</v>
@@ -31102,7 +31102,7 @@
         </is>
       </c>
       <c r="C1708" t="n">
-        <v>0.1469648562300319</v>
+        <v>0</v>
       </c>
       <c r="D1708" t="b">
         <v>0</v>
@@ -31462,7 +31462,7 @@
         </is>
       </c>
       <c r="C1728" t="n">
-        <v>0.0670926517571885</v>
+        <v>0.03973509933774835</v>
       </c>
       <c r="D1728" t="b">
         <v>0</v>
@@ -31606,7 +31606,7 @@
         </is>
       </c>
       <c r="C1736" t="n">
-        <v>0.2268370607028754</v>
+        <v>0.01646090534979424</v>
       </c>
       <c r="D1736" t="b">
         <v>0</v>
@@ -31732,7 +31732,7 @@
         </is>
       </c>
       <c r="C1743" t="n">
-        <v>0.1565495207667732</v>
+        <v>0.02985074626865672</v>
       </c>
       <c r="D1743" t="b">
         <v>0</v>
@@ -31768,7 +31768,7 @@
         </is>
       </c>
       <c r="C1745" t="n">
-        <v>0.1614349775784753</v>
+        <v>0</v>
       </c>
       <c r="D1745" t="b">
         <v>0</v>
@@ -32470,7 +32470,7 @@
         </is>
       </c>
       <c r="C1784" t="n">
-        <v>0.02236421725239617</v>
+        <v>0.009771986970684038</v>
       </c>
       <c r="D1784" t="b">
         <v>0</v>
@@ -32704,7 +32704,7 @@
         </is>
       </c>
       <c r="C1797" t="n">
-        <v>0.05431309904153354</v>
+        <v>0.006756756756756757</v>
       </c>
       <c r="D1797" t="b">
         <v>0</v>
@@ -32740,7 +32740,7 @@
         </is>
       </c>
       <c r="C1799" t="n">
-        <v>0.03194888178913738</v>
+        <v>0.0226537216828479</v>
       </c>
       <c r="D1799" t="b">
         <v>0</v>
@@ -32758,7 +32758,7 @@
         </is>
       </c>
       <c r="C1800" t="n">
-        <v>0.09904153354632587</v>
+        <v>0.007092198581560284</v>
       </c>
       <c r="D1800" t="b">
         <v>0</v>
@@ -33064,7 +33064,7 @@
         </is>
       </c>
       <c r="C1817" t="n">
-        <v>0.03514376996805112</v>
+        <v>0.01954397394136808</v>
       </c>
       <c r="D1817" t="b">
         <v>0</v>
@@ -33208,7 +33208,7 @@
         </is>
       </c>
       <c r="C1825" t="n">
-        <v>0.0926517571884984</v>
+        <v>0.03780068728522337</v>
       </c>
       <c r="D1825" t="b">
         <v>0</v>
@@ -33316,7 +33316,7 @@
         </is>
       </c>
       <c r="C1831" t="n">
-        <v>0.1565495207667732</v>
+        <v>0.03321033210332103</v>
       </c>
       <c r="D1831" t="b">
         <v>0</v>
@@ -33388,10 +33388,10 @@
         </is>
       </c>
       <c r="C1835" t="n">
-        <v>0.6721311475409836</v>
+        <v>0.04901960784313725</v>
       </c>
       <c r="D1835" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="1836">
@@ -33550,7 +33550,7 @@
         </is>
       </c>
       <c r="C1844" t="n">
-        <v>0.02875399361022364</v>
+        <v>0.009900990099009901</v>
       </c>
       <c r="D1844" t="b">
         <v>0</v>
@@ -33730,7 +33730,7 @@
         </is>
       </c>
       <c r="C1854" t="n">
-        <v>0.06389776357827476</v>
+        <v>0.06109324758842444</v>
       </c>
       <c r="D1854" t="b">
         <v>0</v>
@@ -34288,7 +34288,7 @@
         </is>
       </c>
       <c r="C1885" t="n">
-        <v>0.03833865814696485</v>
+        <v>0.01324503311258278</v>
       </c>
       <c r="D1885" t="b">
         <v>0</v>
@@ -34360,7 +34360,7 @@
         </is>
       </c>
       <c r="C1889" t="n">
-        <v>0.08873720136518772</v>
+        <v>0.03676470588235294</v>
       </c>
       <c r="D1889" t="b">
         <v>0</v>
@@ -34468,7 +34468,7 @@
         </is>
       </c>
       <c r="C1895" t="n">
-        <v>0.2109704641350211</v>
+        <v>0.02162162162162162</v>
       </c>
       <c r="D1895" t="b">
         <v>0</v>
@@ -34702,7 +34702,7 @@
         </is>
       </c>
       <c r="C1908" t="n">
-        <v>0.0926517571884984</v>
+        <v>0.003496503496503497</v>
       </c>
       <c r="D1908" t="b">
         <v>0</v>
@@ -34918,7 +34918,7 @@
         </is>
       </c>
       <c r="C1920" t="n">
-        <v>0.1277955271565495</v>
+        <v>0</v>
       </c>
       <c r="D1920" t="b">
         <v>0</v>
@@ -35170,7 +35170,7 @@
         </is>
       </c>
       <c r="C1934" t="n">
-        <v>0.1437699680511182</v>
+        <v>0</v>
       </c>
       <c r="D1934" t="b">
         <v>0</v>
@@ -35458,7 +35458,7 @@
         </is>
       </c>
       <c r="C1950" t="n">
-        <v>0.1261261261261261</v>
+        <v>0.0101010101010101</v>
       </c>
       <c r="D1950" t="b">
         <v>0</v>
@@ -35944,7 +35944,7 @@
         </is>
       </c>
       <c r="C1977" t="n">
-        <v>0.09584664536741214</v>
+        <v>0.003508771929824561</v>
       </c>
       <c r="D1977" t="b">
         <v>0</v>
@@ -36016,7 +36016,7 @@
         </is>
       </c>
       <c r="C1981" t="n">
-        <v>0.02875399361022364</v>
+        <v>0</v>
       </c>
       <c r="D1981" t="b">
         <v>0</v>
@@ -36412,7 +36412,7 @@
         </is>
       </c>
       <c r="C2003" t="n">
-        <v>0.2538860103626943</v>
+        <v>0</v>
       </c>
       <c r="D2003" t="b">
         <v>0</v>
@@ -36808,7 +36808,7 @@
         </is>
       </c>
       <c r="C2025" t="n">
-        <v>0.1405750798722045</v>
+        <v>0</v>
       </c>
       <c r="D2025" t="b">
         <v>0</v>
@@ -36880,7 +36880,7 @@
         </is>
       </c>
       <c r="C2029" t="n">
-        <v>0.08306709265175719</v>
+        <v>0.003460207612456748</v>
       </c>
       <c r="D2029" t="b">
         <v>0</v>
@@ -37024,7 +37024,7 @@
         </is>
       </c>
       <c r="C2037" t="n">
-        <v>0.1309904153354633</v>
+        <v>0</v>
       </c>
       <c r="D2037" t="b">
         <v>0</v>
@@ -37672,7 +37672,7 @@
         </is>
       </c>
       <c r="C2073" t="n">
-        <v>0.421875</v>
+        <v>0</v>
       </c>
       <c r="D2073" t="b">
         <v>0</v>
@@ -37726,7 +37726,7 @@
         </is>
       </c>
       <c r="C2076" t="n">
-        <v>0.3695652173913043</v>
+        <v>0</v>
       </c>
       <c r="D2076" t="b">
         <v>0</v>
@@ -37762,7 +37762,7 @@
         </is>
       </c>
       <c r="C2078" t="n">
-        <v>0.09584664536741214</v>
+        <v>0</v>
       </c>
       <c r="D2078" t="b">
         <v>0</v>
@@ -37798,7 +37798,7 @@
         </is>
       </c>
       <c r="C2080" t="n">
-        <v>0.08306709265175719</v>
+        <v>0</v>
       </c>
       <c r="D2080" t="b">
         <v>0</v>
@@ -37924,7 +37924,7 @@
         </is>
       </c>
       <c r="C2087" t="n">
-        <v>0.1533546325878594</v>
+        <v>0</v>
       </c>
       <c r="D2087" t="b">
         <v>0</v>
@@ -37996,7 +37996,7 @@
         </is>
       </c>
       <c r="C2091" t="n">
-        <v>0.1309904153354633</v>
+        <v>0</v>
       </c>
       <c r="D2091" t="b">
         <v>0</v>
@@ -38320,7 +38320,7 @@
         </is>
       </c>
       <c r="C2109" t="n">
-        <v>0.03514376996805112</v>
+        <v>0.003289473684210526</v>
       </c>
       <c r="D2109" t="b">
         <v>0</v>
@@ -38824,7 +38824,7 @@
         </is>
       </c>
       <c r="C2137" t="n">
-        <v>0.01597444089456869</v>
+        <v>0</v>
       </c>
       <c r="D2137" t="b">
         <v>0</v>
@@ -39256,7 +39256,7 @@
         </is>
       </c>
       <c r="C2161" t="n">
-        <v>0.1076923076923077</v>
+        <v>0.004273504273504274</v>
       </c>
       <c r="D2161" t="b">
         <v>0</v>
@@ -39328,7 +39328,7 @@
         </is>
       </c>
       <c r="C2165" t="n">
-        <v>0.0128755364806867</v>
+        <v>0</v>
       </c>
       <c r="D2165" t="b">
         <v>0</v>
@@ -39940,7 +39940,7 @@
         </is>
       </c>
       <c r="C2199" t="n">
-        <v>0.009584664536741214</v>
+        <v>0</v>
       </c>
       <c r="D2199" t="b">
         <v>0</v>
@@ -40120,7 +40120,7 @@
         </is>
       </c>
       <c r="C2209" t="n">
-        <v>0.0255591054313099</v>
+        <v>0.003257328990228013</v>
       </c>
       <c r="D2209" t="b">
         <v>0</v>
@@ -40696,7 +40696,7 @@
         </is>
       </c>
       <c r="C2241" t="n">
-        <v>0.07028753993610223</v>
+        <v>0</v>
       </c>
       <c r="D2241" t="b">
         <v>0</v>
@@ -40858,7 +40858,7 @@
         </is>
       </c>
       <c r="C2250" t="n">
-        <v>0.05111821086261981</v>
+        <v>0.003344481605351171</v>
       </c>
       <c r="D2250" t="b">
         <v>0</v>
@@ -41524,7 +41524,7 @@
         </is>
       </c>
       <c r="C2287" t="n">
-        <v>0.0926517571884984</v>
+        <v>0.003496503496503497</v>
       </c>
       <c r="D2287" t="b">
         <v>0</v>
@@ -41704,7 +41704,7 @@
         </is>
       </c>
       <c r="C2297" t="n">
-        <v>0.02875399361022364</v>
+        <v>0</v>
       </c>
       <c r="D2297" t="b">
         <v>0</v>
@@ -41794,7 +41794,7 @@
         </is>
       </c>
       <c r="C2302" t="n">
-        <v>0.1950207468879668</v>
+        <v>0</v>
       </c>
       <c r="D2302" t="b">
         <v>0</v>
@@ -41812,7 +41812,7 @@
         </is>
       </c>
       <c r="C2303" t="n">
-        <v>0.1565495207667732</v>
+        <v>0.00749063670411985</v>
       </c>
       <c r="D2303" t="b">
         <v>0</v>
@@ -41938,7 +41938,7 @@
         </is>
       </c>
       <c r="C2310" t="n">
-        <v>0.4025423728813559</v>
+        <v>0.02068965517241379</v>
       </c>
       <c r="D2310" t="b">
         <v>0</v>
@@ -42118,7 +42118,7 @@
         </is>
       </c>
       <c r="C2320" t="n">
-        <v>0.1570247933884298</v>
+        <v>0</v>
       </c>
       <c r="D2320" t="b">
         <v>0</v>
@@ -42298,7 +42298,7 @@
         </is>
       </c>
       <c r="C2330" t="n">
-        <v>0.0926517571884984</v>
+        <v>0</v>
       </c>
       <c r="D2330" t="b">
         <v>0</v>
@@ -42316,7 +42316,7 @@
         </is>
       </c>
       <c r="C2331" t="n">
-        <v>0.03194888178913738</v>
+        <v>0</v>
       </c>
       <c r="D2331" t="b">
         <v>0</v>
@@ -42424,7 +42424,7 @@
         </is>
       </c>
       <c r="C2337" t="n">
-        <v>0.1469648562300319</v>
+        <v>0</v>
       </c>
       <c r="D2337" t="b">
         <v>0</v>
@@ -42532,7 +42532,7 @@
         </is>
       </c>
       <c r="C2343" t="n">
-        <v>0.0670926517571885</v>
+        <v>0</v>
       </c>
       <c r="D2343" t="b">
         <v>0</v>
@@ -43054,7 +43054,7 @@
         </is>
       </c>
       <c r="C2372" t="n">
-        <v>0.0926517571884984</v>
+        <v>0.01384083044982699</v>
       </c>
       <c r="D2372" t="b">
         <v>0</v>
@@ -43666,7 +43666,7 @@
         </is>
       </c>
       <c r="C2406" t="n">
-        <v>0.05431309904153354</v>
+        <v>0</v>
       </c>
       <c r="D2406" t="b">
         <v>0</v>
@@ -43684,7 +43684,7 @@
         </is>
       </c>
       <c r="C2407" t="n">
-        <v>0.008695652173913044</v>
+        <v>0</v>
       </c>
       <c r="D2407" t="b">
         <v>0</v>
@@ -43774,7 +43774,7 @@
         </is>
       </c>
       <c r="C2412" t="n">
-        <v>0.04792332268370607</v>
+        <v>0</v>
       </c>
       <c r="D2412" t="b">
         <v>0</v>
@@ -43828,7 +43828,7 @@
         </is>
       </c>
       <c r="C2415" t="n">
-        <v>0.0743801652892562</v>
+        <v>0</v>
       </c>
       <c r="D2415" t="b">
         <v>0</v>
@@ -43864,7 +43864,7 @@
         </is>
       </c>
       <c r="C2417" t="n">
-        <v>0.009584664536741214</v>
+        <v>0.003205128205128205</v>
       </c>
       <c r="D2417" t="b">
         <v>0</v>
@@ -44008,7 +44008,7 @@
         </is>
       </c>
       <c r="C2425" t="n">
-        <v>0.1246006389776358</v>
+        <v>0</v>
       </c>
       <c r="D2425" t="b">
         <v>0</v>
@@ -44530,7 +44530,7 @@
         </is>
       </c>
       <c r="C2454" t="n">
-        <v>0.0255591054313099</v>
+        <v>0</v>
       </c>
       <c r="D2454" t="b">
         <v>0</v>
@@ -45178,7 +45178,7 @@
         </is>
       </c>
       <c r="C2490" t="n">
-        <v>0.1496062992125984</v>
+        <v>0</v>
       </c>
       <c r="D2490" t="b">
         <v>0</v>
@@ -45340,7 +45340,7 @@
         </is>
       </c>
       <c r="C2499" t="n">
-        <v>0.1565495207667732</v>
+        <v>0.003759398496240601</v>
       </c>
       <c r="D2499" t="b">
         <v>0</v>
@@ -45844,7 +45844,7 @@
         </is>
       </c>
       <c r="C2527" t="n">
-        <v>0.1501597444089457</v>
+        <v>0</v>
       </c>
       <c r="D2527" t="b">
         <v>0</v>
@@ -46040,7 +46040,7 @@
         </is>
       </c>
       <c r="C2538" t="n">
-        <v>0.1533546325878594</v>
+        <v>0</v>
       </c>
       <c r="D2538" t="b">
         <v>0</v>
@@ -46166,7 +46166,7 @@
         </is>
       </c>
       <c r="C2545" t="n">
-        <v>0.2907348242811502</v>
+        <v>0</v>
       </c>
       <c r="D2545" t="b">
         <v>0</v>

</xml_diff>